<commit_message>
changes in key (extra info)
</commit_message>
<xml_diff>
--- a/reference_keys/KEY_PlayInterventionTraining_2.xlsx
+++ b/reference_keys/KEY_PlayInterventionTraining_2.xlsx
@@ -138,6 +138,26 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Key</author>
+  </authors>
+  <commentList>
+    <comment ref="W179" authorId="0" shapeId="0">
+      <text>
+        <t>Coder note: Auto deleted before cake</t>
+      </text>
+    </comment>
+    <comment ref="W244" authorId="0" shapeId="0">
+      <text>
+        <t>Coder note: PLATE was left on screen - didn't code</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3534,7 +3554,7 @@
       </c>
       <c r="W153" t="inlineStr">
         <is>
-          <t>TURTLE - S CANDLE CAKE</t>
+          <t>TURTLE -S CANDLE CAKE</t>
         </is>
       </c>
     </row>
@@ -4024,7 +4044,7 @@
       </c>
       <c r="W179" t="inlineStr">
         <is>
-          <t>DIRTY CANDLE ON CAKE (Auto deleted before cake)</t>
+          <t>DIRTY CANDLE ON CAKE</t>
         </is>
       </c>
     </row>
@@ -5299,7 +5319,7 @@
       </c>
       <c r="W244" t="inlineStr">
         <is>
-          <t>CUP JUICE (PLATE was left on screen-didn't code)</t>
+          <t>CUP JUICE</t>
         </is>
       </c>
     </row>
@@ -7751,5 +7771,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>